<commit_message>
Support static Netlify ZIP with Google-hosted inquiry form and Gmail alerts
</commit_message>
<xml_diff>
--- a/templates/ok-express-customer-list.xlsx
+++ b/templates/ok-express-customer-list.xlsx
@@ -256,7 +256,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Netlify 접수 ID입니다. 중복 처리에 사용하므로 변경하지 마세요.</t>
+        <t>Google 문의 접수 ID입니다. 중복 처리에 사용하므로 변경하지 마세요.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
@@ -30886,7 +30886,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>가져온 Google 시트에서 확장 프로그램 → Apps Script를 열고 저장소의 Code.gs와 manifest를 적용한 뒤 setup을 실행하세요. setup이 본인 Google 이메일을 수신자로 설정합니다.</t>
+          <t>가져온 Google 시트에서 확장 프로그램 → Apps Script를 열고 저장소의 Code.gs와 manifest를 적용한 뒤 setupAndSendTest를 실행하세요. 본인 Google 이메일로 시트 주소가 포함된 테스트 메일을 보냅니다.</t>
         </is>
       </c>
     </row>
@@ -30922,7 +30922,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Google 자동 연동은 Netlify의 GitHub 연결 배포와 Functions 설정이 필요합니다. 정적 ZIP만 업로드해서는 서버 연동 함수가 배포되지 않습니다.</t>
+          <t>Google 자동 연동은 Netlify에는 정적 ZIP을 배포하고, Google Apps Script에 새 Code.gs를 적용해 웹 앱으로 배포합니다. 문의는 Google에서 직접 처리합니다.</t>
         </is>
       </c>
     </row>
@@ -30982,7 +30982,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Netlify 원본, 이사 문의 행, 상담 관리 기록, 이메일, 휴지통과 별도 사본을 함께 관리하세요. Google 버전 기록·백업의 실제 보유 조건도 확인해야 합니다.</t>
+          <t>Google 문의 행, 상담 관리 기록, 이메일, 휴지통과 별도 사본을 함께 관리하세요. Google 버전 기록·백업의 실제 보유 조건도 확인해야 합니다.</t>
         </is>
       </c>
     </row>
@@ -30994,7 +30994,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>사업정보·개인정보 담당자·Google/Netlify 국외이전 안내와 동의, 실제 접수·행 생성·메일 수신을 확인한 뒤 온라인 접수를 여세요.</t>
+          <t>사업정보·개인정보 담당자·Google 처리/국외이전 안내와 동의 및 정적 호스팅 안내를 확정하세요. 새 코드 배포와 시트 저장·메일 수신 확인이 필요합니다.</t>
         </is>
       </c>
     </row>

</xml_diff>